<commit_message>
GTS: rules tab, PJ's capped scoring, team pages, team renaming, reset PIN, promo sound, no personal URL in video
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GTS/printouts/GTS-Pickleball-Offline-Backup.xlsx
+++ b/GTS/printouts/GTS-Pickleball-Offline-Backup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\IAG\GTS\printouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579D05F6-DE86-499D-9467-B412CA664D2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E2C419A-7A1C-4384-9098-A85EDE4D619A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Tie scores turn red. League to 11, semis to 15; above that the winner must lead by 2. Max 21.</t>
+          <t>Tie scores turn red. League: to 11, win by 2, first to 15 wins. Semis: to 15, win by 2, first to 21 wins. Finals: best of 3 games, each like a league game.</t>
         </r>
       </text>
     </comment>
@@ -624,7 +624,7 @@
     <t>4. Finals are best of 3: G1, G2 and (only if 1–1) G3.</t>
   </si>
   <si>
-    <t>Rules: league one game to 11, semis to 15; above the target the winner must lead by 2; max 21.</t>
+    <t>Rules: League to 11, win by 2, first to 15 wins. Semis to 15, win by 2, first to 21 wins. Finals best of 3 games (each to 11, win by 2, first to 15).</t>
   </si>
   <si>
     <t>Generated from the approved Plan B v4 (same times and courts as the website).</t>

</xml_diff>